<commit_message>
Feat: Added new template
</commit_message>
<xml_diff>
--- a/created_tasks.xlsx
+++ b/created_tasks.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,42 +477,452 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2121</v>
+        <v>3270</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reparar manejo de sesiones WebRTC al momento de cerrar un Tab de Sitio o ocurren errores al conectar </t>
+          <t>F1 - Integrar librería OIDC/PKCE</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Flutter - Conexiones WebRTC</t>
+          <t>pubspec.yaml, config/environment.dart</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Reparar manejo de sesiones WebRTC al momento de cerrar un Tab de Sitio o ocurren errores al conectar. Cuando un sitio no ha terminado de conectarse a WebRTC y se cierra, las conexiones quedan abiertas, se debe forzar estos cerrados de conexiones web rtc correctamente cuando se cierra el tab, hay problemas de conexion o se decide desconectarse del sitio.</t>
+          <t>Integrar librería OIDC/PKCE (openid_client/flutter_appauth web) + config entorno</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F2" t="n">
-        <v>2059</v>
+        <v>3269</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Black and Blue\Sprint 57</t>
+          <t>Black and Blue\Sprint 61</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>abdiel.arias@blacknblue.app</t>
+          <t>manuel.betancourt@blacknblue.app</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2025-10-04T16:37:28.29Z</t>
+          <t>2026-06-24T14:45:58.273Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>3271</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>F2 - Lógica de extracción de dominio del email</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>presentation/ui/pages/login/</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Lógica de extracción de dominio del email (debounce on-change / on-submit del campo correo)</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>3269</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Black and Blue\Sprint 61</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>manuel.betancourt@blacknblue.app</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-06-24T14:46:06.48Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3272</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>F3 - Datasource: checkSsoDomain(email)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>infrastructure/datasources/authentication/</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Datasource: checkSsoDomain(email) → GET /auth/sso/discovery</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" t="n">
+        <v>3269</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Black and Blue\Sprint 61</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>manuel.betancourt@blacknblue.app</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-06-24T14:46:14.023Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3273</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>F4 - UI condicional: dominio OKTA</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>login_page.dart</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>UI condicional: si dominio = OKTA → mostrar botón "Iniciar sesión con Okta" y ocultar campo password; si no → login tradicional</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" t="n">
+        <v>3269</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Black and Blue\Sprint 61</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>manuel.betancourt@blacknblue.app</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-06-24T14:46:21.81Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3274</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>F5 - Iniciar flujo Auth Code + PKCE</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>presentation/, datasource</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Iniciar flujo Auth Code + PKCE (generar state/code_verifier/nonce, redirigir a OKTA del site)</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" t="n">
+        <v>3269</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Black and Blue\Sprint 61</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>manuel.betancourt@blacknblue.app</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-06-24T14:46:29.617Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>3275</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>F6 - Página /auth/callback</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>presentation/router/, nueva página</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Página /auth/callback: validar state, intercambio code→token, validar nonce; registrar ruta en router</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>6</v>
+      </c>
+      <c r="F7" t="n">
+        <v>3269</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Black and Blue\Sprint 61</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>manuel.betancourt@blacknblue.app</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-06-24T14:46:37.28Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>3276</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>F7 - Datasource loginWithOkta</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>infrastructure/datasources/authentication/</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Datasource loginWithOkta(idToken, siteId) → POST /users/auth/okta → AuthUserResponse</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>3269</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Black and Blue\Sprint 61</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>manuel.betancourt@blacknblue.app</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-06-24T14:46:45.27Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>3277</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>F8 - Conectar al BLoC/guardado de sesión</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>presentation/blocs/auth_user_bloc/</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Conectar al BLoC/guardado de sesión actual (reuso, sin cambios al BLoC)</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3269</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Black and Blue\Sprint 61</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>manuel.betancourt@blacknblue.app</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-06-24T14:46:53.787Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>3278</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>F9 - Manejo de errores UX</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>login_page.dart</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Manejo de errores UX (dominio inactivo, token inválido, email no verificado, usuario rechazado)</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" t="n">
+        <v>3269</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Black and Blue\Sprint 61</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>manuel.betancourt@blacknblue.app</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-06-24T14:47:00.613Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>3279</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>F10 - UI gestionar dominios OKTA (opcional admin)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>presentation/ui/pages/</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>(Opcional admin) UI para gestionar dominios OKTA por site</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3269</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Black and Blue\Sprint 61</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>manuel.betancourt@blacknblue.app</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-06-24T14:47:06.99Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>3280</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>F11 - Tests widget/integración</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>test/</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Tests widget/integración (discovery muestra botón, flujo callback)</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>6</v>
+      </c>
+      <c r="F12" t="n">
+        <v>3269</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Black and Blue\Sprint 61</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>manuel.betancourt@blacknblue.app</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-06-24T14:47:15.347Z</t>
         </is>
       </c>
     </row>

</xml_diff>